<commit_message>
feat: add ambassador and communication dashboard prompt
</commit_message>
<xml_diff>
--- a/pss-2.0-global/.claude/screen-tracker/SCREEN-STATUS-OVERVIEW.xlsx
+++ b/pss-2.0-global/.claude/screen-tracker/SCREEN-STATUS-OVERVIEW.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repos\PWDS\pwds-soruban\pss-2.0-global\.claude\screen-tracker\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repos\PWDS\pwds-soruban - Copy\pss-2.0-global\.claude\screen-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1300" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1318" uniqueCount="246">
   <si>
     <t>Screen #</t>
   </si>
@@ -1073,7 +1073,106 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="28">
+  <dxfs count="37">
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE0E7FF"/>
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE0E7FF"/>
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE0E7FF"/>
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE0E7FF"/>
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF4B5563"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF3F4F6"/>
+          <bgColor rgb="FFF3F4F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF854D0E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEF9C3"/>
+          <bgColor rgb="FFFEF9C3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDBEAFE"/>
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEF3C7"/>
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCFCE7"/>
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF3730A3"/>
@@ -4998,8 +5097,8 @@
       <c r="G107" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H107" s="5" t="s">
-        <v>17</v>
+      <c r="H107" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="I107" s="2" t="s">
         <v>16</v>
@@ -5025,8 +5124,11 @@
       <c r="E108" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F108" s="6" t="s">
-        <v>18</v>
+      <c r="F108" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G108" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="H108" s="6" t="s">
         <v>18</v>
@@ -5051,8 +5153,11 @@
       <c r="E109" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F109" s="6" t="s">
-        <v>18</v>
+      <c r="F109" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G109" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="H109" s="6" t="s">
         <v>18</v>
@@ -5104,7 +5209,10 @@
         <v>32</v>
       </c>
       <c r="F111" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G111" t="s">
+        <v>16</v>
       </c>
       <c r="H111" s="6" t="s">
         <v>18</v>
@@ -5442,7 +5550,10 @@
         <v>32</v>
       </c>
       <c r="F124" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G124" t="s">
+        <v>16</v>
       </c>
       <c r="H124" s="6" t="s">
         <v>18</v>
@@ -5468,7 +5579,10 @@
         <v>32</v>
       </c>
       <c r="F125" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G125" t="s">
+        <v>16</v>
       </c>
       <c r="H125" s="6" t="s">
         <v>18</v>
@@ -5494,7 +5608,10 @@
         <v>32</v>
       </c>
       <c r="F126" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G126" t="s">
+        <v>16</v>
       </c>
       <c r="H126" s="6" t="s">
         <v>18</v>
@@ -5520,7 +5637,10 @@
         <v>32</v>
       </c>
       <c r="F127" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G127" t="s">
+        <v>16</v>
       </c>
       <c r="H127" s="6" t="s">
         <v>18</v>
@@ -5546,7 +5666,10 @@
         <v>32</v>
       </c>
       <c r="F128" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G128" t="s">
+        <v>16</v>
       </c>
       <c r="H128" s="6" t="s">
         <v>18</v>
@@ -5572,7 +5695,10 @@
         <v>32</v>
       </c>
       <c r="F129" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G129" t="s">
+        <v>16</v>
       </c>
       <c r="H129" s="6" t="s">
         <v>18</v>
@@ -5598,7 +5724,10 @@
         <v>32</v>
       </c>
       <c r="F130" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G130" t="s">
+        <v>16</v>
       </c>
       <c r="H130" s="6" t="s">
         <v>18</v>
@@ -5624,7 +5753,10 @@
         <v>32</v>
       </c>
       <c r="F131" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G131" t="s">
+        <v>16</v>
       </c>
       <c r="H131" s="6" t="s">
         <v>18</v>
@@ -5650,7 +5782,10 @@
         <v>32</v>
       </c>
       <c r="F132" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G132" t="s">
+        <v>16</v>
       </c>
       <c r="H132" s="6" t="s">
         <v>18</v>
@@ -5676,7 +5811,10 @@
         <v>32</v>
       </c>
       <c r="F133" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G133" t="s">
+        <v>16</v>
       </c>
       <c r="H133" s="6" t="s">
         <v>18</v>
@@ -5702,7 +5840,10 @@
         <v>32</v>
       </c>
       <c r="F134" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G134" t="s">
+        <v>16</v>
       </c>
       <c r="H134" s="6" t="s">
         <v>18</v>
@@ -5728,7 +5869,10 @@
         <v>32</v>
       </c>
       <c r="F135" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G135" t="s">
+        <v>16</v>
       </c>
       <c r="H135" s="6" t="s">
         <v>18</v>
@@ -5754,7 +5898,10 @@
         <v>32</v>
       </c>
       <c r="F136" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G136" t="s">
+        <v>16</v>
       </c>
       <c r="H136" s="6" t="s">
         <v>18</v>
@@ -5780,7 +5927,10 @@
         <v>32</v>
       </c>
       <c r="F137" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G137" t="s">
+        <v>16</v>
       </c>
       <c r="H137" s="6" t="s">
         <v>18</v>
@@ -5806,7 +5956,10 @@
         <v>32</v>
       </c>
       <c r="F138" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="G138" t="s">
+        <v>16</v>
       </c>
       <c r="H138" s="6" t="s">
         <v>18</v>
@@ -6181,108 +6334,137 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E152">
-    <cfRule type="cellIs" dxfId="27" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="10" operator="equal">
       <formula>"High"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="11" operator="equal">
       <formula>"Medium"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="12" operator="equal">
       <formula>"Low"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F152">
-    <cfRule type="cellIs" dxfId="24" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="13" operator="equal">
       <formula>"Completed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="23" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="14" operator="equal">
       <formula>"Completed - Needs Fix"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="15" operator="equal">
       <formula>"Ready to Build"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="16" operator="equal">
       <formula>"In Progress (Partial)"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="17" operator="equal">
       <formula>"Not Started"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="18" operator="equal">
       <formula>"Upcoming (Dashboard)"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="19" operator="equal">
       <formula>"Upcoming (Config)"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="20" operator="equal">
       <formula>"Upcoming (Mobile)"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="21" operator="equal">
       <formula>"Upcoming"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H152">
-    <cfRule type="cellIs" dxfId="15" priority="13" operator="equal">
+  <conditionalFormatting sqref="H2:H106 H108:H152">
+    <cfRule type="cellIs" dxfId="24" priority="22" operator="equal">
       <formula>"Not Started"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="23" operator="equal">
       <formula>"Pending"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="24" operator="equal">
       <formula>"In Testing"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="25" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="26" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="27" operator="equal">
       <formula>"Issues Found"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="28" operator="equal">
       <formula>"Blocked - Awaiting Fix"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="29" operator="equal">
       <formula>"N/A (Upcoming)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J152">
-    <cfRule type="cellIs" dxfId="7" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="30" operator="equal">
       <formula>"Not Started"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="31" operator="equal">
       <formula>"Pending"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="32" operator="equal">
       <formula>"In Testing"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="33" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="25" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="34" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="35" operator="equal">
       <formula>"Issues Found"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="27" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="36" operator="equal">
       <formula>"Blocked - Awaiting Fix"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="28" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="37" operator="equal">
       <formula>"N/A (Upcoming)"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H107">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+      <formula>"Completed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+      <formula>"Completed - Needs Fix"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+      <formula>"Ready to Build"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
+      <formula>"In Progress (Partial)"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+      <formula>"Not Started"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="6" operator="equal">
+      <formula>"Upcoming (Dashboard)"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="7" operator="equal">
+      <formula>"Upcoming (Config)"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="8" operator="equal">
+      <formula>"Upcoming (Mobile)"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="9" operator="equal">
+      <formula>"Upcoming"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" sqref="E2:E152">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F152">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F152 H107">
       <formula1>"Completed,Completed - Needs Fix,Ready to Build,In Progress (Partial),Not Started,Upcoming (Dashboard),Upcoming (Config),Upcoming (Mobile),Upcoming"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G2:G152 I2:I152 K2:K152">
+    <dataValidation type="list" allowBlank="1" sqref="K2:K152 I2:I152 G2:G152">
       <formula1>"Karthick,Saranya,Kavin,Sangeetha"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H2:H152 J2:J152">
+    <dataValidation type="list" allowBlank="1" sqref="J2:J152 H2:H106 H108:H152">
       <formula1>"Not Started,Pending,In Testing,Passed,Failed,Issues Found,Blocked - Awaiting Fix,N/A (Upcoming)"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6455,7 +6637,7 @@
       </c>
       <c r="B5" s="17">
         <f>COUNTIF('Screen Status'!F2:F152,"Completed")</f>
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="C5" s="18">
         <f>COUNTIF('Screen Status'!F2:F152,"Completed - Needs Fix")</f>
@@ -6471,7 +6653,7 @@
       </c>
       <c r="F5" s="21">
         <f>COUNTIF('Screen Status'!F2:F152,"Not Started")</f>
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="G5" s="22">
         <f>COUNTIF('Screen Status'!F2:F152,"Upcoming*")</f>
@@ -6577,7 +6759,7 @@
       </c>
       <c r="B10" s="28">
         <f>COUNTIFS('Screen Status'!B2:B152,"Administration",'Screen Status'!F2:F152,"Completed")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10" s="28">
         <f>COUNTIFS('Screen Status'!B2:B152,"Administration",'Screen Status'!F2:F152,"Completed - Needs Fix")</f>
@@ -6593,7 +6775,7 @@
       </c>
       <c r="F10" s="28">
         <f>COUNTIFS('Screen Status'!B2:B152,"Administration",'Screen Status'!F2:F152,"Not Started")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G10" s="28">
         <f>COUNTIFS('Screen Status'!B2:B152,"Administration",'Screen Status'!F2:F152,"Upcoming (Dashboard)")</f>
@@ -6712,7 +6894,7 @@
       </c>
       <c r="B13" s="28">
         <f>COUNTIFS('Screen Status'!B2:B152,"Contacts",'Screen Status'!F2:F152,"Completed")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C13" s="28">
         <f>COUNTIFS('Screen Status'!B2:B152,"Contacts",'Screen Status'!F2:F152,"Completed - Needs Fix")</f>
@@ -6728,7 +6910,7 @@
       </c>
       <c r="F13" s="28">
         <f>COUNTIFS('Screen Status'!B2:B152,"Contacts",'Screen Status'!F2:F152,"Not Started")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" s="28">
         <f>COUNTIFS('Screen Status'!B2:B152,"Contacts",'Screen Status'!F2:F152,"Upcoming (Dashboard)")</f>
@@ -6802,7 +6984,7 @@
       </c>
       <c r="B15" s="28">
         <f>COUNTIFS('Screen Status'!B2:B152,"Fundraising",'Screen Status'!F2:F152,"Completed")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C15" s="28">
         <f>COUNTIFS('Screen Status'!B2:B152,"Fundraising",'Screen Status'!F2:F152,"Completed - Needs Fix")</f>
@@ -6818,7 +7000,7 @@
       </c>
       <c r="F15" s="28">
         <f>COUNTIFS('Screen Status'!B2:B152,"Fundraising",'Screen Status'!F2:F152,"Not Started")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G15" s="28">
         <f>COUNTIFS('Screen Status'!B2:B152,"Fundraising",'Screen Status'!F2:F152,"Upcoming (Dashboard)")</f>
@@ -7207,7 +7389,7 @@
       </c>
       <c r="B24" s="29">
         <f>COUNTIF('Screen Status'!F2:F152,"Completed")</f>
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="C24" s="29">
         <f>COUNTIF('Screen Status'!F2:F152,"Completed - Needs Fix")</f>
@@ -7223,7 +7405,7 @@
       </c>
       <c r="F24" s="29">
         <f>COUNTIF('Screen Status'!F2:F152,"Not Started")</f>
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="G24" s="29">
         <f>COUNTIF('Screen Status'!F2:F152,"Upcoming (Dashboard)")</f>
@@ -7590,7 +7772,7 @@
       </c>
       <c r="C32" s="28">
         <f>COUNTIFS('Screen Status'!B2:B152,"Contacts",'Screen Status'!H2:H152,"Pending")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D32" s="28">
         <f>COUNTIFS('Screen Status'!B2:B152,"Contacts",'Screen Status'!H2:H152,"In Testing")</f>
@@ -8349,7 +8531,7 @@
       </c>
       <c r="C43" s="29">
         <f>COUNTIF('Screen Status'!H2:H152,"Pending")</f>
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D43" s="29">
         <f>COUNTIF('Screen Status'!H2:H152,"In Testing")</f>
@@ -8436,7 +8618,7 @@
       </c>
       <c r="B47" s="28">
         <f>COUNTIFS('Screen Status'!E2:E152,"High",'Screen Status'!F2:F152,"Completed")</f>
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C47" s="28">
         <f>COUNTIFS('Screen Status'!E2:E152,"High",'Screen Status'!F2:F152,"In Progress (Partial)")</f>
@@ -8444,7 +8626,7 @@
       </c>
       <c r="D47" s="28">
         <f>COUNTIF('Screen Status'!E2:E152,"High")-COUNTIFS('Screen Status'!E2:E152,"High",'Screen Status'!F2:F152,"Completed")-COUNTIFS('Screen Status'!E2:E152,"High",'Screen Status'!F2:F152,"In Progress (Partial)")</f>
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E47" s="29">
         <f>COUNTIF('Screen Status'!E2:E152,"High")</f>
@@ -8457,7 +8639,7 @@
       </c>
       <c r="B48" s="28">
         <f>COUNTIFS('Screen Status'!E2:E152,"Medium",'Screen Status'!F2:F152,"Completed")</f>
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C48" s="28">
         <f>COUNTIFS('Screen Status'!E2:E152,"Medium",'Screen Status'!F2:F152,"In Progress (Partial)")</f>
@@ -8465,7 +8647,7 @@
       </c>
       <c r="D48" s="28">
         <f>COUNTIF('Screen Status'!E2:E152,"Medium")-COUNTIFS('Screen Status'!E2:E152,"Medium",'Screen Status'!F2:F152,"Completed")-COUNTIFS('Screen Status'!E2:E152,"Medium",'Screen Status'!F2:F152,"In Progress (Partial)")</f>
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E48" s="29">
         <f>COUNTIF('Screen Status'!E2:E152,"Medium")</f>
@@ -8539,7 +8721,7 @@
       </c>
       <c r="B53" s="28">
         <f>COUNTIFS('Screen Status'!G2:G152,"Karthick",'Screen Status'!F2:F152,"Completed")+COUNTIFS('Screen Status'!G2:G152,"Karthick",'Screen Status'!F2:F152,"Completed - Needs Fix")</f>
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="C53" s="28">
         <f>COUNTIFS('Screen Status'!I2:I152,"Karthick",'Screen Status'!H2:H152,"Passed")</f>
@@ -8555,7 +8737,7 @@
       </c>
       <c r="F53" s="28">
         <f>COUNTIFS('Screen Status'!I2:I152,"Karthick",'Screen Status'!H2:H152,"Pending")+COUNTIFS('Screen Status'!I2:I152,"Karthick",'Screen Status'!H2:H152,"Not Started")+COUNTIFS('Screen Status'!I2:I152,"Karthick",'Screen Status'!H2:H152,"In Testing")+COUNTIFS('Screen Status'!I2:I152,"Karthick",'Screen Status'!H2:H152,"Blocked - Awaiting Fix")</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G53" s="28">
         <f>COUNTIFS('Screen Status'!K2:K152,"Karthick",'Screen Status'!J2:J152,"Passed")</f>
@@ -8575,7 +8757,7 @@
       </c>
       <c r="K53" s="29">
         <f>SUM(B53:J53)</f>
-        <v>63</v>
+        <v>80</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.3">

</xml_diff>